<commit_message>
Updated and grouped learning activities and media types
</commit_message>
<xml_diff>
--- a/Training Designer Blank Template.xlsx
+++ b/Training Designer Blank Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kevin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a376289e25d8d65e/Projects/training-designer/training-designer-vanilla/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E6D5D05-1F2C-4373-A8CA-D4E24D15955D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9132" yWindow="3180" windowWidth="30936" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Training Program" sheetId="1" r:id="rId1"/>
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="90">
   <si>
     <t>Day</t>
   </si>
@@ -342,57 +342,27 @@
     <t>Self-Paced</t>
   </si>
   <si>
-    <t>eLearning</t>
-  </si>
-  <si>
     <t>Apply</t>
   </si>
   <si>
     <t>On-the-Job Training</t>
   </si>
   <si>
-    <t>Cognitive Tasks</t>
-  </si>
-  <si>
-    <t>Delivery Methods</t>
-  </si>
-  <si>
-    <t>Watching</t>
-  </si>
-  <si>
     <t>Evaluate</t>
   </si>
   <si>
-    <t>Listening</t>
-  </si>
-  <si>
     <t>Microlearning</t>
   </si>
   <si>
-    <t>Procedural - Customer Service</t>
-  </si>
-  <si>
     <t>Create</t>
   </si>
   <si>
-    <t>Navigation Practice</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>Web Article</t>
-  </si>
-  <si>
     <t>Documentation Practice</t>
   </si>
   <si>
-    <t>Problem-Solving - Customer Service</t>
-  </si>
-  <si>
-    <t>Interactive Q&amp;A</t>
-  </si>
-  <si>
     <t>Recorded Lecture</t>
   </si>
   <si>
@@ -408,148 +378,193 @@
     <t>Knowledge Check</t>
   </si>
   <si>
-    <t>Activity Sheets</t>
-  </si>
-  <si>
     <t>Collaborative Platform</t>
   </si>
   <si>
-    <t>VR/AR</t>
-  </si>
-  <si>
     <t>Live Customer Practice</t>
   </si>
   <si>
-    <t>Game</t>
-  </si>
-  <si>
-    <t>Workshop</t>
-  </si>
-  <si>
     <t>Link</t>
   </si>
   <si>
     <t>Scenario-Based Exercise</t>
   </si>
   <si>
-    <t>Graded Mock Calls</t>
-  </si>
-  <si>
-    <t>Navigation Assessment</t>
+    <t>Text Document</t>
+  </si>
+  <si>
+    <t>Spreadsheet</t>
+  </si>
+  <si>
+    <t>Live Group Discussion</t>
+  </si>
+  <si>
+    <t>Asynchronous Group Discussion</t>
+  </si>
+  <si>
+    <t>Written Graded Assessment</t>
+  </si>
+  <si>
+    <t>Peer Assessment</t>
+  </si>
+  <si>
+    <t>Self Assessment</t>
+  </si>
+  <si>
+    <t>Discussion Channel</t>
+  </si>
+  <si>
+    <t>Plan</t>
+  </si>
+  <si>
+    <t>Keep</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>Rebrand</t>
+  </si>
+  <si>
+    <t>Minor Change</t>
+  </si>
+  <si>
+    <t>Major Update</t>
+  </si>
+  <si>
+    <t>Merge w/ Below</t>
+  </si>
+  <si>
+    <t>Add to Above</t>
+  </si>
+  <si>
+    <t>Split</t>
+  </si>
+  <si>
+    <t>New Addition</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Unit (Main Topic)</t>
+  </si>
+  <si>
+    <t>Module (Subtopic)</t>
+  </si>
+  <si>
+    <t>Content Type</t>
+  </si>
+  <si>
+    <t>Facts / Concepts</t>
+  </si>
+  <si>
+    <t>Video / Recording Review</t>
+  </si>
+  <si>
+    <t>Workflow - Operations / Admin / Support</t>
+  </si>
+  <si>
+    <t>Activity Sheet / Workbook</t>
+  </si>
+  <si>
+    <t>Procedural - Software / Tools</t>
+  </si>
+  <si>
+    <t>Podcast / Audio Review</t>
+  </si>
+  <si>
+    <t>Online Article / Web Page</t>
+  </si>
+  <si>
+    <t>Procedural - Communication Skills</t>
+  </si>
+  <si>
+    <t>eLearning - Read, Watch, Listen</t>
+  </si>
+  <si>
+    <t>Problem-Solving - Software / Tools</t>
+  </si>
+  <si>
+    <t>eLearning - Interactive</t>
+  </si>
+  <si>
+    <t>Infographic / Visual Aid</t>
+  </si>
+  <si>
+    <t>Problem-Solving - Communication Skills</t>
+  </si>
+  <si>
+    <t>Q&amp;A with Instructor / Expert</t>
+  </si>
+  <si>
+    <t>Audio Recording / Podcast</t>
+  </si>
+  <si>
+    <t>Recap &amp; Debrief</t>
+  </si>
+  <si>
+    <t>Facilitated Group Activity</t>
+  </si>
+  <si>
+    <t>eLearning Module</t>
+  </si>
+  <si>
+    <t>Concept Mapping / Mind Mapping</t>
+  </si>
+  <si>
+    <t>Quiz / Survey</t>
+  </si>
+  <si>
+    <t>Pre-Training / Advance Organizer</t>
+  </si>
+  <si>
+    <t>Live System / Application</t>
+  </si>
+  <si>
+    <t>Worked Example Review</t>
+  </si>
+  <si>
+    <t>Digital Workspace / Notebook</t>
+  </si>
+  <si>
+    <t>eLearning - Simulate &amp; Practice</t>
+  </si>
+  <si>
+    <t>Software / Tool Practice</t>
+  </si>
+  <si>
+    <t>Guest Speaker / SME Session</t>
+  </si>
+  <si>
+    <t>Job Aid &amp; Reference Lookup Practice</t>
+  </si>
+  <si>
+    <t>VR / AR</t>
+  </si>
+  <si>
+    <t>Shadowing &amp; Job Observation</t>
+  </si>
+  <si>
+    <t>Role Play / Mock Conversation</t>
+  </si>
+  <si>
+    <t>Mentorship / Coaching</t>
+  </si>
+  <si>
+    <t>Procedural Skills Assessment</t>
+  </si>
+  <si>
+    <t>Graded Practice Conversation</t>
+  </si>
+  <si>
+    <t>Learning Game</t>
   </si>
   <si>
     <t>Meet &amp; Greet</t>
   </si>
   <si>
-    <t>Text Document</t>
-  </si>
-  <si>
-    <t>Spreadsheet</t>
-  </si>
-  <si>
-    <t>Graphics</t>
-  </si>
-  <si>
-    <t>Subject Matter Expert</t>
-  </si>
-  <si>
-    <t>Procedural - Software/ Tools</t>
-  </si>
-  <si>
-    <t>Workflow - Operations/ Admin/ Support</t>
-  </si>
-  <si>
-    <t>Problem-Solving - Software/ Tools</t>
-  </si>
-  <si>
-    <t>Audio Recording/ Podcast</t>
-  </si>
-  <si>
-    <t>Quiz/ Survey</t>
-  </si>
-  <si>
-    <t>Tool/ Software</t>
-  </si>
-  <si>
-    <t>Mentorship/ Coaching</t>
-  </si>
-  <si>
-    <t>Shadowing/ Observation</t>
-  </si>
-  <si>
-    <t>Role Play/ Mock Call Exercise</t>
-  </si>
-  <si>
-    <t>Recap/ Debrief</t>
-  </si>
-  <si>
-    <t>Reference/ Job Aids Practice</t>
-  </si>
-  <si>
-    <t>Module Interaction</t>
-  </si>
-  <si>
-    <t>Live Group Discussion</t>
-  </si>
-  <si>
-    <t>Asynchronous Group Discussion</t>
-  </si>
-  <si>
-    <t>Written Graded Assessment</t>
-  </si>
-  <si>
-    <t>Peer Assessment</t>
-  </si>
-  <si>
-    <t>Self Assessment</t>
-  </si>
-  <si>
-    <t>Facts/ Concepts</t>
-  </si>
-  <si>
-    <t>Discussion Channel</t>
-  </si>
-  <si>
-    <t>Online Notebook</t>
-  </si>
-  <si>
-    <t>Plan</t>
-  </si>
-  <si>
-    <t>Keep</t>
-  </si>
-  <si>
-    <t>Remove</t>
-  </si>
-  <si>
-    <t>Rebrand</t>
-  </si>
-  <si>
-    <t>Minor Change</t>
-  </si>
-  <si>
-    <t>Major Update</t>
-  </si>
-  <si>
-    <t>Merge w/ Below</t>
-  </si>
-  <si>
-    <t>Add to Above</t>
-  </si>
-  <si>
-    <t>Split</t>
-  </si>
-  <si>
-    <t>New Addition</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Unit (Main Topic)</t>
-  </si>
-  <si>
-    <t>Module (Subtopic)</t>
+    <t>Ice Breaker</t>
   </si>
 </sst>
 </file>
@@ -615,6 +630,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -953,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>83</v>
+        <v>50</v>
       </c>
       <c r="C1" t="s">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -980,13 +999,13 @@
         <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="L1" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
       <c r="M1" t="s">
-        <v>82</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1022,17 +1041,17 @@
           </x14:formula1>
           <xm:sqref>E2:E300</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{6E809DD4-F105-4BA1-93E2-6CF60566103F}">
-          <x14:formula1>
-            <xm:f>Options!$B$2:$B$29</xm:f>
-          </x14:formula1>
-          <xm:sqref>F2:F300</xm:sqref>
-        </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BC7BDF5D-D1C6-4D31-A02B-2BA345CDA32B}">
           <x14:formula1>
             <xm:f>Options!$F$2:$F$10</xm:f>
           </x14:formula1>
           <xm:sqref>L2:L300</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{65FB8312-6A7B-4ADE-AE91-BF16055E82C0}">
+          <x14:formula1>
+            <xm:f>Options!$B$2:$B$35</xm:f>
+          </x14:formula1>
+          <xm:sqref>F2:F1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1042,35 +1061,35 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.69921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.19921875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.19921875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.8984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.59765625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.3984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.59765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
         <v>3</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="D1" t="s">
         <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="F1" t="s">
-        <v>72</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
@@ -1084,13 +1103,13 @@
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="F2" t="s">
-        <v>73</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -1098,503 +1117,647 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
         <v>16</v>
       </c>
-      <c r="B4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>60</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>79</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F9" t="s">
-        <v>80</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>81</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>34</v>
+        <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F11" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F13" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" t="s">
+        <v>77</v>
+      </c>
+      <c r="C15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D15" t="s">
         <v>27</v>
       </c>
-      <c r="B15" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" t="s">
-        <v>70</v>
-      </c>
       <c r="E15" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F15" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>78</v>
       </c>
       <c r="C16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>71</v>
+        <v>38</v>
       </c>
       <c r="E16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D17" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="E17" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F18" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D19" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E19" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F19" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>83</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D20" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F20" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E21" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F21" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="C22" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="D22" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>34</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
       </c>
       <c r="D23" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E23" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F23" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
       <c r="B24" t="s">
-        <v>68</v>
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
       </c>
       <c r="D24" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F24" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
       <c r="B25" t="s">
-        <v>59</v>
+        <v>28</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
       </c>
       <c r="D25" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F25" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
       <c r="B26" t="s">
-        <v>40</v>
+        <v>84</v>
+      </c>
+      <c r="C26" t="s">
+        <v>20</v>
       </c>
       <c r="D26" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E26" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F26" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>20</v>
+      </c>
       <c r="B27" t="s">
-        <v>58</v>
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
       </c>
       <c r="D27" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F27" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>20</v>
+      </c>
       <c r="B28" t="s">
-        <v>41</v>
+        <v>37</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
       </c>
       <c r="D28" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F28" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>20</v>
+      </c>
       <c r="B29" t="s">
-        <v>47</v>
+        <v>36</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
       </c>
       <c r="D29" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="E29" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F29" t="s">
-        <v>27</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" t="s">
+        <v>20</v>
+      </c>
+      <c r="E30" t="s">
+        <v>20</v>
+      </c>
+      <c r="F30" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>20</v>
+      </c>
+      <c r="B32" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>20</v>
+      </c>
+      <c r="B33" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" t="s">
+        <v>20</v>
+      </c>
+      <c r="E33" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" t="s">
+        <v>20</v>
+      </c>
+      <c r="E34" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B35" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1 A7:A22 C19:C22 C17:C18 C1" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated layout of charts and tables in report section
</commit_message>
<xml_diff>
--- a/Training Designer Blank Template.xlsx
+++ b/Training Designer Blank Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a376289e25d8d65e/Projects/training-designer/training-designer-vanilla/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E6D5D05-1F2C-4373-A8CA-D4E24D15955D}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C21C98BC-6B1C-45CC-835A-90C1CA84B937}"/>
   <bookViews>
-    <workbookView xWindow="9132" yWindow="3180" windowWidth="30936" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Training Program" sheetId="1" r:id="rId1"/>
@@ -295,7 +295,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="90">
   <si>
     <t>Day</t>
   </si>
@@ -1097,13 +1097,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
         <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s">
         <v>53</v>
@@ -1117,13 +1117,13 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>54</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
         <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s">
         <v>55</v>
@@ -1137,13 +1137,13 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
         <v>57</v>
@@ -1157,13 +1157,13 @@
         <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
         <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
         <v>60</v>
@@ -1177,13 +1177,13 @@
         <v>19</v>
       </c>
       <c r="B6" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
         <v>20</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
         <v>62</v>
@@ -1197,13 +1197,13 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
         <v>20</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="E7" t="s">
         <v>65</v>
@@ -1217,7 +1217,7 @@
         <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
@@ -1237,13 +1237,13 @@
         <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
         <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
         <v>20</v>
@@ -1257,13 +1257,13 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C10" t="s">
         <v>20</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s">
         <v>20</v>
@@ -1277,13 +1277,13 @@
         <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
         <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E11" t="s">
         <v>20</v>
@@ -1297,13 +1297,13 @@
         <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
         <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
         <v>20</v>
@@ -1317,7 +1317,7 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
         <v>20</v>
@@ -1337,13 +1337,13 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="C14" t="s">
         <v>20</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E14" t="s">
         <v>20</v>
@@ -1377,7 +1377,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C16" t="s">
         <v>20</v>
@@ -1397,7 +1397,7 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>82</v>
       </c>
       <c r="C17" t="s">
         <v>20</v>
@@ -1417,7 +1417,7 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C18" t="s">
         <v>20</v>
@@ -1437,7 +1437,7 @@
         <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="C19" t="s">
         <v>20</v>
@@ -1457,7 +1457,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>34</v>
       </c>
       <c r="C20" t="s">
         <v>20</v>
@@ -1477,7 +1477,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C21" t="s">
         <v>20</v>
@@ -1517,7 +1517,7 @@
         <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>34</v>
+        <v>84</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
@@ -1557,7 +1557,7 @@
         <v>20</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>83</v>
       </c>
       <c r="C25" t="s">
         <v>20</v>
@@ -1577,7 +1577,7 @@
         <v>20</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="C26" t="s">
         <v>20</v>
@@ -1597,7 +1597,7 @@
         <v>20</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="C27" t="s">
         <v>20</v>
@@ -1617,7 +1617,7 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="C28" t="s">
         <v>20</v>
@@ -1677,7 +1677,7 @@
         <v>20</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C31" t="s">
         <v>20</v>
@@ -1697,7 +1697,7 @@
         <v>20</v>
       </c>
       <c r="B32" t="s">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="C32" t="s">
         <v>20</v>
@@ -1717,7 +1717,7 @@
         <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
         <v>20</v>
@@ -1737,7 +1737,7 @@
         <v>20</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C34" t="s">
         <v>20</v>
@@ -1754,7 +1754,10 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+      <c r="D35" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
shifted from SheetsJS to ExcelJS
</commit_message>
<xml_diff>
--- a/Training Designer Blank Template.xlsx
+++ b/Training Designer Blank Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a376289e25d8d65e/Projects/training-designer/training-designer-vanilla/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C21C98BC-6B1C-45CC-835A-90C1CA84B937}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{05B440BE-26B7-4700-AC98-1554B011D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD948801-1A29-4430-8D12-4542E3569862}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20544" yWindow="0" windowWidth="20832" windowHeight="16656" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Training Program" sheetId="1" r:id="rId1"/>
@@ -20,282 +20,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Tabora, Kevin (Operations &amp; Technology)</author>
-  </authors>
-  <commentList>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{7FB35097-320D-4E36-BFE0-5C081F1F7E4A}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Main topic that groups related content together</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{13CF2E68-0BF1-4788-93C8-4CD89333AD39}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Specific subject within the chapter</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{84921801-A244-48C2-B804-5BF3953D60F6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Clear statement of what learners should be able to do after completion</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{3492F690-7F8D-4134-9396-BD49995CAC24}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-The type of thinking skills required</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="0" shapeId="0" xr:uid="{B2F1E068-8591-4FA6-BD0F-46C3FBB8C2F5}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-How learners will engage with the content</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G1" authorId="0" shapeId="0" xr:uid="{17DDDABA-74BF-4104-971F-BD0EAA514D83}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-The instructional approach used to structure learning experiences</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0" shapeId="0" xr:uid="{67EEF79C-C13A-4DE5-ACC1-665FD52CC5C6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-The physical or digital formats used to present content</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{52BA7F35-10EB-433B-AA71-D1B68A29FA15}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Category of information being taught</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0" shapeId="0" xr:uid="{5956F65F-B4E9-4543-828A-0468F884A82F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Minutes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K1" authorId="0" shapeId="0" xr:uid="{3FD18B41-ADBE-4FD0-BC00-1F776F0E3BE4}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Ensure the link starts with http:// or https://</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L1" authorId="0" shapeId="0" xr:uid="{FB1FEE22-88EB-4BA1-B61C-88496FA61A95}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Tabora, Kevin (Operations &amp; Technology):</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-Indicates intended changes to existing training</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="89">
   <si>
     <t>Day</t>
   </si>
@@ -313,9 +39,6 @@
   </si>
   <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>Type of Content</t>
   </si>
   <si>
     <t>Duration</t>
@@ -571,26 +294,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -957,7 +667,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M1"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
@@ -972,10 +682,10 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C1" t="s">
         <v>50</v>
-      </c>
-      <c r="C1" t="s">
-        <v>51</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
@@ -993,27 +703,26 @@
         <v>5</v>
       </c>
       <c r="I1" t="s">
+        <v>51</v>
+      </c>
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
-        <v>7</v>
-      </c>
       <c r="K1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="M1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1 D1:I1" numberStoredAsText="1"/>
+    <ignoredError sqref="A1 D1:H1" numberStoredAsText="1"/>
   </ignoredErrors>
-  <legacyDrawing r:id="rId1"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="6">
@@ -1086,678 +795,678 @@
         <v>5</v>
       </c>
       <c r="E1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
-        <v>21</v>
-      </c>
       <c r="C14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F24" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F28" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F29" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B31" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F31" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B32" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F32" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B34" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F34" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D35" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>